<commit_message>
Add automatic group-stage scheduling and knockout bracket generation
Admin now uploads just a team roster (division/group/team/players);
the app auto-generates the round-robin schedule within each group,
computes live standings (wins, point diff, head-to-head/mini-league
tiebreaks), and lets the admin generate a seeded knockout bracket
(with byes) once group play is confirmed. Knockout winners advance
into the next round automatically. Replaces the old fully-manual,
pre-built-bracket upload flow.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample-bracket.xlsx
+++ b/fixtures/sample-bracket.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="대진표" sheetId="1" r:id="rId1"/>
+    <sheet name="명단" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,38 +397,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>수준</v>
       </c>
       <c r="B1" t="str">
-        <v>라운드</v>
+        <v>조</v>
       </c>
       <c r="C1" t="str">
-        <v>코트</v>
+        <v>팀명</v>
       </c>
       <c r="D1" t="str">
-        <v>경기순서</v>
+        <v>선수1</v>
       </c>
       <c r="E1" t="str">
-        <v>팀A명</v>
-      </c>
-      <c r="F1" t="str">
-        <v>A선수1</v>
-      </c>
-      <c r="G1" t="str">
-        <v>A선수2</v>
-      </c>
-      <c r="H1" t="str">
-        <v>팀B명</v>
-      </c>
-      <c r="I1" t="str">
-        <v>B선수1</v>
-      </c>
-      <c r="J1" t="str">
-        <v>B선수2</v>
+        <v>선수2</v>
       </c>
     </row>
     <row r="2">
@@ -436,31 +421,16 @@
         <v>3.0</v>
       </c>
       <c r="B2" t="str">
-        <v>1라운드</v>
+        <v>A</v>
       </c>
       <c r="C2" t="str">
-        <v>1코트</v>
+        <v>번개조</v>
       </c>
       <c r="D2" t="str">
-        <v>1</v>
+        <v>김철수</v>
       </c>
       <c r="E2" t="str">
-        <v>번개조</v>
-      </c>
-      <c r="F2" t="str">
-        <v>김철수</v>
-      </c>
-      <c r="G2" t="str">
         <v>이영희</v>
-      </c>
-      <c r="H2" t="str">
-        <v>천둥조</v>
-      </c>
-      <c r="I2" t="str">
-        <v>박민수</v>
-      </c>
-      <c r="J2" t="str">
-        <v>최지은</v>
       </c>
     </row>
     <row r="3">
@@ -468,31 +438,16 @@
         <v>3.0</v>
       </c>
       <c r="B3" t="str">
-        <v>1라운드</v>
+        <v>A</v>
       </c>
       <c r="C3" t="str">
-        <v>2코트</v>
+        <v>구름조</v>
       </c>
       <c r="D3" t="str">
-        <v>2</v>
+        <v>정다솔</v>
       </c>
       <c r="E3" t="str">
-        <v>구름조</v>
-      </c>
-      <c r="F3" t="str">
-        <v>정다솔</v>
-      </c>
-      <c r="G3" t="str">
         <v>한가람</v>
-      </c>
-      <c r="H3" t="str">
-        <v>번개조</v>
-      </c>
-      <c r="I3" t="str">
-        <v>김철수</v>
-      </c>
-      <c r="J3" t="str">
-        <v>이영희</v>
       </c>
     </row>
     <row r="4">
@@ -500,63 +455,33 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="str">
-        <v>2라운드</v>
+        <v>A</v>
       </c>
       <c r="C4" t="str">
-        <v>1코트</v>
+        <v>천둥조</v>
       </c>
       <c r="D4" t="str">
-        <v>3</v>
+        <v>박민수</v>
       </c>
       <c r="E4" t="str">
-        <v>천둥조</v>
-      </c>
-      <c r="F4" t="str">
-        <v>박민수</v>
-      </c>
-      <c r="G4" t="str">
         <v>최지은</v>
-      </c>
-      <c r="H4" t="str">
-        <v>구름조</v>
-      </c>
-      <c r="I4" t="str">
-        <v>정다솔</v>
-      </c>
-      <c r="J4" t="str">
-        <v>한가람</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="B5" t="str">
-        <v>결승</v>
+        <v>A</v>
       </c>
       <c r="C5" t="str">
-        <v>1코트</v>
+        <v>독수리조</v>
       </c>
       <c r="D5" t="str">
-        <v>4</v>
+        <v>이수민</v>
       </c>
       <c r="E5" t="str">
-        <v>번개조</v>
-      </c>
-      <c r="F5" t="str">
-        <v>김철수</v>
-      </c>
-      <c r="G5" t="str">
-        <v>이영희오타</v>
-      </c>
-      <c r="H5" t="str">
-        <v>구름조</v>
-      </c>
-      <c r="I5" t="str">
-        <v>정다솔</v>
-      </c>
-      <c r="J5" t="str">
-        <v>한가람</v>
+        <v>장하나</v>
       </c>
     </row>
     <row r="6">
@@ -564,30 +489,15 @@
         <v>3.5</v>
       </c>
       <c r="B6" t="str">
-        <v>1라운드</v>
+        <v>A</v>
       </c>
       <c r="C6" t="str">
-        <v>1코트</v>
+        <v>매화조</v>
       </c>
       <c r="D6" t="str">
-        <v>1</v>
+        <v>오세훈</v>
       </c>
       <c r="E6" t="str">
-        <v>독수리조</v>
-      </c>
-      <c r="F6" t="str">
-        <v>이수민</v>
-      </c>
-      <c r="G6" t="str">
-        <v>장하나</v>
-      </c>
-      <c r="H6" t="str">
-        <v>매화조</v>
-      </c>
-      <c r="I6" t="str">
-        <v>오세훈</v>
-      </c>
-      <c r="J6" t="str">
         <v>윤도현</v>
       </c>
     </row>
@@ -596,68 +506,21 @@
         <v>3.5</v>
       </c>
       <c r="B7" t="str">
-        <v>1라운드</v>
+        <v>A</v>
       </c>
       <c r="C7" t="str">
-        <v>2코트</v>
+        <v>소나무조</v>
       </c>
       <c r="D7" t="str">
-        <v>2</v>
+        <v>배소연</v>
       </c>
       <c r="E7" t="str">
-        <v>소나무조</v>
-      </c>
-      <c r="F7" t="str">
-        <v>배소연</v>
-      </c>
-      <c r="G7" t="str">
-        <v>임재현</v>
-      </c>
-      <c r="H7" t="str">
-        <v>독수리조</v>
-      </c>
-      <c r="I7" t="str">
-        <v>이수민</v>
-      </c>
-      <c r="J7" t="str">
-        <v>장하나</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>3.5</v>
-      </c>
-      <c r="B8" t="str">
-        <v>2라운드</v>
-      </c>
-      <c r="C8" t="str">
-        <v>1코트</v>
-      </c>
-      <c r="D8" t="str">
-        <v>3</v>
-      </c>
-      <c r="E8" t="str">
-        <v>매화조</v>
-      </c>
-      <c r="F8" t="str">
-        <v>오세훈</v>
-      </c>
-      <c r="G8" t="str">
-        <v>윤도현</v>
-      </c>
-      <c r="H8" t="str">
-        <v>소나무조</v>
-      </c>
-      <c r="I8" t="str">
-        <v>배소연</v>
-      </c>
-      <c r="J8" t="str">
         <v>임재현</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove 팀명 (team name) as a manual roster input field
Rosters now only need 부문, 조, 선수1, 선수2 — the display team name
is auto-generated from the two player names (e.g. "김철수·이영희")
instead of being typed in separately, for both xlsx/csv upload and
the admin single-team-add form. Updates the fixture templates and
upload instructions to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample-bracket.xlsx
+++ b/fixtures/sample-bracket.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="명단" sheetId="1" r:id="rId1"/>
+    <sheet name="팀 명단" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,12 +407,9 @@
         <v>조</v>
       </c>
       <c r="C1" t="str">
-        <v>팀명</v>
+        <v>선수1</v>
       </c>
       <c r="D1" t="str">
-        <v>선수1</v>
-      </c>
-      <c r="E1" t="str">
         <v>선수2</v>
       </c>
     </row>
@@ -424,12 +421,9 @@
         <v>A</v>
       </c>
       <c r="C2" t="str">
-        <v>번개조</v>
+        <v>김철수</v>
       </c>
       <c r="D2" t="str">
-        <v>김철수</v>
-      </c>
-      <c r="E2" t="str">
         <v>이영희</v>
       </c>
     </row>
@@ -441,12 +435,9 @@
         <v>A</v>
       </c>
       <c r="C3" t="str">
-        <v>구름조</v>
+        <v>정다솔</v>
       </c>
       <c r="D3" t="str">
-        <v>정다솔</v>
-      </c>
-      <c r="E3" t="str">
         <v>한가람</v>
       </c>
     </row>
@@ -458,12 +449,9 @@
         <v>A</v>
       </c>
       <c r="C4" t="str">
-        <v>천둥조</v>
+        <v>박민수</v>
       </c>
       <c r="D4" t="str">
-        <v>박민수</v>
-      </c>
-      <c r="E4" t="str">
         <v>최지은</v>
       </c>
     </row>
@@ -475,12 +463,9 @@
         <v>A</v>
       </c>
       <c r="C5" t="str">
-        <v>독수리조</v>
+        <v>이수민</v>
       </c>
       <c r="D5" t="str">
-        <v>이수민</v>
-      </c>
-      <c r="E5" t="str">
         <v>장하나</v>
       </c>
     </row>
@@ -492,12 +477,9 @@
         <v>A</v>
       </c>
       <c r="C6" t="str">
-        <v>매화조</v>
+        <v>오세훈</v>
       </c>
       <c r="D6" t="str">
-        <v>오세훈</v>
-      </c>
-      <c r="E6" t="str">
         <v>윤도현</v>
       </c>
     </row>
@@ -509,18 +491,15 @@
         <v>A</v>
       </c>
       <c r="C7" t="str">
-        <v>소나무조</v>
+        <v>배소연</v>
       </c>
       <c r="D7" t="str">
-        <v>배소연</v>
-      </c>
-      <c r="E7" t="str">
         <v>임재현</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>